<commit_message>
Run #5 Pass 2: Indiana complete (170 courses). Updated tracker and COURSE_EXPANSION.md.
</commit_message>
<xml_diff>
--- a/data/Chains Course Catalog.xlsx
+++ b/data/Chains Course Catalog.xlsx
@@ -579,11 +579,11 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Partial</t>
+          <t>DONE</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>150</v>
+        <v>170</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -595,12 +595,12 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Pass 1: top 150 of 169 PDGA×DGS cross-verified courses (318 DGS-listed total). 19 verified remain — finish next pass.</t>
+          <t>Complete: 150 pass 1 + 20 pass 2 = 170 total. No per-hole data (option d); users add pars in-app.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Data Scout run #8: sync WI row with GitHub state (1→69 OSM recovery)
</commit_message>
<xml_diff>
--- a/data/Chains Course Catalog.xlsx
+++ b/data/Chains Course Catalog.xlsx
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>150</v>
+        <v>315</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -557,12 +557,12 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Pass 1 of ~3: top 150 of 283 PDGA×DGS cross-verified courses (443 DGS-listed total). Continue next pass.</t>
+          <t>Pass 1+2: 165 + 150 new = 315 total. 66 pass 2 geocoded; 84 pending. Pass 3: ~14 remain of 329 PDGA-listed.</t>
         </is>
       </c>
     </row>
@@ -621,11 +621,11 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>70</v>
+        <v>30</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>None (0/70) — no compliant public per-hole source; users add pars in-app</t>
+          <t>None (0/30)</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -633,12 +633,12 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Pass 1 of ~3: top 70 of 393 DiscGolfScene-listed courses. Geo: city centroid. Continue next pass.</t>
+          <t>Pass 1 rebuild: 30 OSM courses recovered (original 70 lost). ~363 remain.</t>
         </is>
       </c>
     </row>
@@ -653,16 +653,31 @@
           <t>thin - revisit</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Revisit - state filter issue; found: 4-H Camp Riversite (Hingham)</t>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>69</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>None (0/69) — no compliant public per-hole source; users add pars in-app</t>
         </is>
       </c>
       <c r="F6" t="n">
         <v>5</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-07-31</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Pass 1: OSM Overpass (69 courses, precise lat/lng). ~50-100+ remain via PDGA cross-check (needs JS rendering).</t>
+        </is>
       </c>
     </row>
     <row r="7">

</xml_diff>

<commit_message>
Data Scout run #13 — OH tracker update: 270/315 geocoded
</commit_message>
<xml_diff>
--- a/data/Chains Course Catalog.xlsx
+++ b/data/Chains Course Catalog.xlsx
@@ -545,7 +545,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>315</v>
+        <v>270</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -562,7 +562,7 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Pass 1+2: 165 + 150 new = 315 total. 66 pass 2 geocoded; 84 pending. Pass 3: ~14 remain of 329 PDGA-listed.</t>
+          <t>270/315 geocoded (85%); 45 small-town gaps remain. Geocoding pass 3 via Nominatim (top 8 cities).</t>
         </is>
       </c>
     </row>

</xml_diff>